<commit_message>
feat: Toshi overhaul, LarAgent activation, onboarding fixes, school data seed + full dashboard audit
- Fixed confirmYes/confirmNo button routing (callStepHandler bypasses send())
- Fixed commitAll for complete mode (added students/subjects, idempotent inserts)
- Fixed WhatsApp skip, mount restoreState, post-commit assistant mode
- Fixed updatedAttachment  ->  (fee/exam upload crash)
- Fixed Calendar/Events Vue errors (this.date.end, prop/data conflict)
- Fixed Settings 404s (created missing logo/favicon images)
- Fixed Toshi header layout (extra </div> tags from refactor)
- Fixed MRR query (wrong status: active -> approve)
- Renamed Reports -> Data Exports across all dashboards
- Added mode dropdown (Claude-style) with slash commands
- Added shared Blade partials (mode dropdown, skip button)
- Enabled TOSHI_LARAGENT_ENABLED with 3 new tools
- Seeded Test School One: 32 students, 9 teachers, 8 parents, 7 exams, 65 marks
- Full Playwright audit: 18 sections, 0 console errors
</commit_message>
<xml_diff>
--- a/public/templates/exam-upload-template.xlsx
+++ b/public/templates/exam-upload-template.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -507,76 +507,44 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Term I</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Midterm</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Primary 1</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Mathematics</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>John Ssali</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>End of Term 1</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Term I</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>End of Term</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Primary 2</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Jane Okello</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Mid Term 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>End of Term 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Mock Exam</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>End of Term 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Final Exam</t>
         </is>
       </c>
     </row>

</xml_diff>